<commit_message>
Add shared-formula reconstruction on read
Excel's shared-formula optimization (its default when filling/dragging a
formula across a range) only stores expression text on the group's master
cell; other cells in the group carried just a cached value and were read
back with an empty formula. Reader now reconstructs each cell's own formula
by shifting the master's unanchored references by the cell offset, the same
way Excel itself expands the group.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/SafeOpenXml.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/SafeOpenXml.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R53ab894cc2f842cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3f980e2a34404902"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raf54b3fe526b4a22"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dc7942a124b4d64"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R763c1e7c108543c6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R92735f920e064f41"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85db9379d2fc496d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fda3fdf9a204880"/>
 </x:worksheet>
 </file>
</xml_diff>